<commit_message>
chore(ag): add filtering and settings for rpg2 autofilter
</commit_message>
<xml_diff>
--- a/django/camac/statistics/config/kt_ag/rpg2_export.xlsx
+++ b/django/camac/statistics/config/kt_ag/rpg2_export.xlsx
@@ -623,20 +623,18 @@
       <c r="A6" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B6" cm="1">
-        <f t="array" ref="B6">SUM(SUMIFS(Flächen!D:D,Flächen!E:E,{"Beton";"Andere wasserundurchlässige Beläge (z.B. Asphalt)"},Flächen!G:G,{"Erschliessung, Verkehr (kommunale und private Projekte)","Ausnahmebewilligung Artikel 24ff RPG","Andere"}))</f>
-        <v>0</v>
+      <c r="B6">
+        <f>SUBTOTAL(109,Flächen!$D:$D)</f>
+        <v/>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B7" cm="1">
-        <f t="array" ref="B7">SUM(SUMIFS(Dossiers!$D:$D,Dossiers!$H:$H,"Ja",Dossiers!$I:$I,{"Ja",""}))
--SUM(SUMIFS(Dossiers!$E:$E,Dossiers!$H:$H,"Ja",Dossiers!$I:$I,{"Ja",""}))
--SUM(SUMIFS(Dossiers!$F:$F,Dossiers!$H:$H,"Ja",Dossiers!$I:$I,{"Ja",""}))</f>
-        <v>0</v>
+      <c r="B7">
+        <f>SUBTOTAL(109,Dossiers!$D:$D)-SUBTOTAL(109,Dossiers!$E:$E)-SUBTOTAL(109,Dossiers!$F:$F)</f>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>